<commit_message>
Complete Milestones 3 and 4 with integration and documentation
</commit_message>
<xml_diff>
--- a/agile_documents/Unit_Test_Plan.xlsx
+++ b/agile_documents/Unit_Test_Plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vijay\OneDrive\Desktop\AI-Project-Intelligence-Risk-Advisor\agile_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF010466-A85D-4875-B5C9-71D77ADE0FDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B720A7DE-FD05-40CC-8D94-F549641368FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C3B83BB6-2AB9-4547-8541-9F6969E92BF1}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="210">
   <si>
     <t>Actual Result</t>
   </si>
@@ -283,6 +283,387 @@
   </si>
   <si>
     <t>All three agents executed successfully and the combined validation completed successfully with “MILESTONE 2 VALIDATION COMPLETED.”</t>
+  </si>
+  <si>
+    <t>Documentation Generation Agent</t>
+  </si>
+  <si>
+    <t>Run the Documentation Generation Agent using the uploaded project document knowledge base.</t>
+  </si>
+  <si>
+    <t>Project documents containing project activities and requirements are available.</t>
+  </si>
+  <si>
+    <t>Documentation Generation Agent should successfully generate structured project documentation.</t>
+  </si>
+  <si>
+    <t>Documentation generated successfully.</t>
+  </si>
+  <si>
+    <t>User Story Generation</t>
+  </si>
+  <si>
+    <t>Run the Documentation Generation Agent and generate User Stories from the project documents.</t>
+  </si>
+  <si>
+    <t>Project documents contain information about project activities, requirements, or work items.</t>
+  </si>
+  <si>
+    <t>User Stories should be generated in a structured format using only information supported by the project documents.</t>
+  </si>
+  <si>
+    <t>User Stories successfully generated in the required structured format.</t>
+  </si>
+  <si>
+    <t>Risk Register Generation</t>
+  </si>
+  <si>
+    <t>Run the Documentation Generation Agent and generate a Risk Register from the project documents.</t>
+  </si>
+  <si>
+    <t>Project documents contain information about identified project risks.</t>
+  </si>
+  <si>
+    <t>A structured Risk Register should be generated containing supported risk information such as description, impact, likelihood, risk level, and mitigation.</t>
+  </si>
+  <si>
+    <t>Risk Register successfully generated using the available project information.</t>
+  </si>
+  <si>
+    <t>Action Item Generation</t>
+  </si>
+  <si>
+    <t>Run the Documentation Generation Agent and generate structured Action Items.</t>
+  </si>
+  <si>
+    <t>Project documents contain pending or required project actions.</t>
+  </si>
+  <si>
+    <t>Structured Action Items should be generated with responsibility, priority, and status when explicitly available.</t>
+  </si>
+  <si>
+    <t>Action Items successfully generated from the project documents.</t>
+  </si>
+  <si>
+    <t>Documentation Missing Information Handling</t>
+  </si>
+  <si>
+    <t>Run the Documentation Generation Agent when some documentation details are unavailable in the project documents.</t>
+  </si>
+  <si>
+    <t>Impact, likelihood, mitigation, responsibility, priority, or status information is unavailable.</t>
+  </si>
+  <si>
+    <t>Missing information should be reported as not specified in the documents without inventing project information.</t>
+  </si>
+  <si>
+    <t>Project Health Scoring</t>
+  </si>
+  <si>
+    <t>Run the Project Health Scoring module using the uploaded project documents.</t>
+  </si>
+  <si>
+    <t>Project documents are available for health assessment.</t>
+  </si>
+  <si>
+    <t>Project Health Scoring should generate an overall project health score based on document evidence.</t>
+  </si>
+  <si>
+    <t>Project health assessment generated successfully.</t>
+  </si>
+  <si>
+    <t>Scope Clarity Scoring</t>
+  </si>
+  <si>
+    <t>Run the Project Health Scoring module and evaluate Scope Clarity.</t>
+  </si>
+  <si>
+    <t>Project documents contain information about project goals, deliverables, and scope.</t>
+  </si>
+  <si>
+    <t>Scope Clarity score should be generated from 0 to 100 with supporting evidence.</t>
+  </si>
+  <si>
+    <t>Scope Clarity score successfully generated with supporting evidence.</t>
+  </si>
+  <si>
+    <t>Timeline Risk Scoring</t>
+  </si>
+  <si>
+    <t>Run the Project Health Scoring module and evaluate Timeline Risk.</t>
+  </si>
+  <si>
+    <t>Project documents contain project status, schedule, risks, or delay information.</t>
+  </si>
+  <si>
+    <t>Timeline Risk score should be generated from 0 to 100 and supported by project evidence.</t>
+  </si>
+  <si>
+    <t>Timeline Risk score successfully generated with supporting evidence.</t>
+  </si>
+  <si>
+    <t>Blocker Count Assessment</t>
+  </si>
+  <si>
+    <t>Run the Project Health Scoring module and identify documented blockers.</t>
+  </si>
+  <si>
+    <t>Project documents may contain current blockers or may contain no explicit blockers.</t>
+  </si>
+  <si>
+    <t>Documented blockers should be identified and counted; if none are explicitly documented, the system should report that no explicit blockers were found.</t>
+  </si>
+  <si>
+    <t>Blocker assessment successfully generated and documented blockers correctly reported.</t>
+  </si>
+  <si>
+    <t>Overall Project Health Assessment</t>
+  </si>
+  <si>
+    <t>Execute the complete Project Health Scoring module.</t>
+  </si>
+  <si>
+    <t>Scope Clarity, Timeline Risk, and blocker information are available from the project documents.</t>
+  </si>
+  <si>
+    <t>Overall project health score should be generated from 0 to 100 with an explanation based on the available evidence.</t>
+  </si>
+  <si>
+    <t>Overall project health score successfully generated with evidence-based assessment.</t>
+  </si>
+  <si>
+    <t>Conversational Project Assistant</t>
+  </si>
+  <si>
+    <t>Ask a project-related question through the Conversational Project Intelligence Assistant.</t>
+  </si>
+  <si>
+    <t>Uploaded project documents are available in the RAG knowledge base.</t>
+  </si>
+  <si>
+    <t>Assistant should retrieve relevant project information and provide a response based on the uploaded documents.</t>
+  </si>
+  <si>
+    <t>Project-related question answered successfully using the uploaded project documents.</t>
+  </si>
+  <si>
+    <t>Document-Grounded Question Answering</t>
+  </si>
+  <si>
+    <t>Ask the assistant a question whose answer is available in the uploaded project documents.</t>
+  </si>
+  <si>
+    <t>Relevant information is present in the project knowledge base.</t>
+  </si>
+  <si>
+    <t>Assistant should provide a relevant answer based only on the retrieved project-document evidence.</t>
+  </si>
+  <si>
+    <t>Relevant answer successfully generated from the uploaded project documents.</t>
+  </si>
+  <si>
+    <t>Unrelated Question Protection</t>
+  </si>
+  <si>
+    <t>Ask the assistant an unrelated general-knowledge question that is not supported by the uploaded project documents.</t>
+  </si>
+  <si>
+    <t>Requested information is not available in the project documents.</t>
+  </si>
+  <si>
+    <t>Assistant should not provide an unrelated general-knowledge answer and should respond that the information is not specified in the uploaded project documents.</t>
+  </si>
+  <si>
+    <t>Unrelated question correctly rejected with the expected document-information message.</t>
+  </si>
+  <si>
+    <t>Conversational Assistant Missing Information Handling</t>
+  </si>
+  <si>
+    <t>Ask the assistant a project-related question for which information is not available in the uploaded documents.</t>
+  </si>
+  <si>
+    <t>Required project information is not specified in the project documents.</t>
+  </si>
+  <si>
+    <t>Assistant should report that the information is not specified in the uploaded project documents without inventing information.</t>
+  </si>
+  <si>
+    <t>Missing project information correctly reported as not specified in the uploaded project documents.</t>
+  </si>
+  <si>
+    <t>Combined Milestone 3 Validation</t>
+  </si>
+  <si>
+    <t>Execute the combined Milestone 3 validation covering Documentation Generation, Project Health Scoring, and Conversational Project Intelligence Assistant.</t>
+  </si>
+  <si>
+    <t>All Milestone 3 modules and the RAG knowledge base are available.</t>
+  </si>
+  <si>
+    <t>Documentation Generation, Project Health Scoring, and Conversational Assistant should execute successfully and produce document-grounded project intelligence.</t>
+  </si>
+  <si>
+    <t>All three Milestone 3 components executed successfully and the combined validation was completed successfully.</t>
+  </si>
+  <si>
+    <t>Integrated Application Workflow</t>
+  </si>
+  <si>
+    <t>Launch the Streamlit application and access the main project intelligence features.</t>
+  </si>
+  <si>
+    <t>All required application modules and dependencies are available.</t>
+  </si>
+  <si>
+    <t>End-to-End Document Processing</t>
+  </si>
+  <si>
+    <t>Upload a supported project document and process it through ingestion, chunking, embedding generation, and vector indexing.</t>
+  </si>
+  <si>
+    <t>A valid project document is available.</t>
+  </si>
+  <si>
+    <t>Document Retrieval Validation</t>
+  </si>
+  <si>
+    <t>Upload a project document and ask a question about information contained in it.</t>
+  </si>
+  <si>
+    <t>Relevant information exists in the indexed document.</t>
+  </si>
+  <si>
+    <t>Multi-Agent Integration</t>
+  </si>
+  <si>
+    <t>Execute the Scope, Risk and Delivery Forecasting, and Blocker and Action Item Identification agents.</t>
+  </si>
+  <si>
+    <t>The RAG pipeline and all three agents are available.</t>
+  </si>
+  <si>
+    <t>Documentation Generation Integration</t>
+  </si>
+  <si>
+    <t>Generate User Stories, a Risk Register, and Action Items through the integrated application.</t>
+  </si>
+  <si>
+    <t>Relevant project information is available in uploaded documents.</t>
+  </si>
+  <si>
+    <t>Project Health Integration</t>
+  </si>
+  <si>
+    <t>Run the Project Health Scoring module through the integrated application.</t>
+  </si>
+  <si>
+    <t>Project documents contain information suitable for health assessment.</t>
+  </si>
+  <si>
+    <t>Conversational Assistant Integration</t>
+  </si>
+  <si>
+    <t>Ask a project-related question through the application interface.</t>
+  </si>
+  <si>
+    <t>The assistant and document retrieval pipeline are available.</t>
+  </si>
+  <si>
+    <t>Unsupported File Handling</t>
+  </si>
+  <si>
+    <t>Upload a file format that is not supported by the application.</t>
+  </si>
+  <si>
+    <t>An unsupported file is provided.</t>
+  </si>
+  <si>
+    <t>Empty or Missing Document Information</t>
+  </si>
+  <si>
+    <t>Ask a question about information that is not available in the uploaded documents.</t>
+  </si>
+  <si>
+    <t>The requested information is absent from the document knowledge base.</t>
+  </si>
+  <si>
+    <t>Document Processing Error Handling</t>
+  </si>
+  <si>
+    <t>Test the processing workflow with an invalid, unreadable, or otherwise unsuitable input file.</t>
+  </si>
+  <si>
+    <t>The input cannot be processed successfully.</t>
+  </si>
+  <si>
+    <t>LLM Provider Fallback</t>
+  </si>
+  <si>
+    <t>Simulate a failure or unavailability of the primary LLM provider and execute a supported request.</t>
+  </si>
+  <si>
+    <t>A fallback provider is configured and available.</t>
+  </si>
+  <si>
+    <t>Project Health Display Validation</t>
+  </si>
+  <si>
+    <t>Open the project health interface and inspect the displayed indicators and score.</t>
+  </si>
+  <si>
+    <t>The health assessment has generated results.</t>
+  </si>
+  <si>
+    <t>README and Milestone Documentation Review</t>
+  </si>
+  <si>
+    <t>Review README.md and MILESTONE_4.md against the implemented application and project structure.</t>
+  </si>
+  <si>
+    <t>Both documentation files are present.</t>
+  </si>
+  <si>
+    <t>The application should launch successfully and provide access to the integrated features.</t>
+  </si>
+  <si>
+    <t>Pending validation</t>
+  </si>
+  <si>
+    <t>The document should be processed and indexed successfully.</t>
+  </si>
+  <si>
+    <t>The retrieval pipeline should return relevant information from the uploaded document.</t>
+  </si>
+  <si>
+    <t>The agents should execute and generate their respective structured project intelligence outputs.</t>
+  </si>
+  <si>
+    <t>Structured project documentation should be generated using supported document evidence.</t>
+  </si>
+  <si>
+    <t>The application should display the implemented health indicators and overall score.</t>
+  </si>
+  <si>
+    <t>The assistant should return a relevant response grounded in available project documents.</t>
+  </si>
+  <si>
+    <t>The application should handle the file appropriately and provide suitable feedback.</t>
+  </si>
+  <si>
+    <t>The application should report that the information is not specified rather than inventing details.</t>
+  </si>
+  <si>
+    <t>The application should handle the error appropriately without an uncontrolled failure.</t>
+  </si>
+  <si>
+    <t>The application should use the configured fallback mechanism or report the failure clearly.</t>
+  </si>
+  <si>
+    <t>The displayed indicators and score should correspond to the calculated assessment.</t>
+  </si>
+  <si>
+    <t>Documentation should accurately describe the project features, setup, and Milestone 4 scope.</t>
   </si>
 </sst>
 </file>
@@ -323,7 +704,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -346,26 +727,47 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -681,21 +1083,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF95B16C-182C-4757-B929-A728708A2DB0}">
-  <dimension ref="A1:J18"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J46"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.1796875" customWidth="1"/>
-    <col min="2" max="2" width="14.26953125" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="5" width="16.54296875" customWidth="1"/>
-    <col min="6" max="6" width="15.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.1796875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="14.26953125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="15" style="4" customWidth="1"/>
+    <col min="4" max="5" width="16.54296875" style="4" customWidth="1"/>
+    <col min="6" max="6" width="15.81640625" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="8.7265625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="31" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:10" s="3" customFormat="1" ht="31" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -711,345 +1114,905 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="77.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="93" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="93" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="4"/>
-    </row>
-    <row r="4" spans="1:10" ht="77.5" x14ac:dyDescent="0.25">
+      <c r="J3" s="5"/>
+    </row>
+    <row r="4" spans="1:10" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="93" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="93" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="93" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="93" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="93" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="93" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="77.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="139.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="139.5" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="139.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="139.5" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="124" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="124" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="108.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="124" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="124" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="124" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="124" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="124" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="124" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="108.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="108.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="217" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="217" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="2" t="s">
         <v>82</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="139.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="155" x14ac:dyDescent="0.35">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="201.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="139.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="155" x14ac:dyDescent="0.35">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="124" x14ac:dyDescent="0.35">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="124" x14ac:dyDescent="0.35">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="108.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="201.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="139.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="139.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="139.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="217" x14ac:dyDescent="0.35">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="170.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="201.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="124" x14ac:dyDescent="0.35">
+      <c r="A34" s="8">
+        <v>33</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="186" x14ac:dyDescent="0.35">
+      <c r="A35" s="8">
+        <v>34</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="139.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="8">
+        <v>35</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="139.5" x14ac:dyDescent="0.35">
+      <c r="A37" s="8">
+        <v>36</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="139.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="8">
+        <v>37</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="108.5" x14ac:dyDescent="0.35">
+      <c r="A39" s="8">
+        <v>38</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="124" x14ac:dyDescent="0.35">
+      <c r="A40" s="8">
+        <v>39</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="108.5" x14ac:dyDescent="0.35">
+      <c r="A41" s="8">
+        <v>40</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="124" x14ac:dyDescent="0.35">
+      <c r="A42" s="8">
+        <v>41</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="124" x14ac:dyDescent="0.35">
+      <c r="A43" s="8">
+        <v>42</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="124" x14ac:dyDescent="0.35">
+      <c r="A44" s="8">
+        <v>43</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="108.5" x14ac:dyDescent="0.35">
+      <c r="A45" s="8">
+        <v>44</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="155" x14ac:dyDescent="0.35">
+      <c r="A46" s="8">
+        <v>45</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>